<commit_message>
ajustes para acoplar el pipeline  de cada variable a la carga manual de datos desde la interfaz
</commit_message>
<xml_diff>
--- a/Descripcion_fuentes.xlsx
+++ b/Descripcion_fuentes.xlsx
@@ -2990,8 +2990,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010072D1BA84C54EAF45AC5884A45A375563" ma:contentTypeVersion="7" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="22c1915734ddaa8afa723c2fd2af65c9">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="909962d2-3dca-4f1f-a40d-c5b9a956a4cc" xmlns:ns3="2ec83a8d-0db2-4f0a-a71c-c237315b29ff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d0850c7b2b411963c54362962e5a3bc3" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010072D1BA84C54EAF45AC5884A45A375563" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e7d927febeb335f2d1c85a73b8edbe09">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="909962d2-3dca-4f1f-a40d-c5b9a956a4cc" xmlns:ns3="2ec83a8d-0db2-4f0a-a71c-c237315b29ff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="26a6144809e82f96be1dd4a023cacbb7" ns2:_="" ns3:_="">
     <xsd:import namespace="909962d2-3dca-4f1f-a40d-c5b9a956a4cc"/>
     <xsd:import namespace="2ec83a8d-0db2-4f0a-a71c-c237315b29ff"/>
     <xsd:element name="properties">
@@ -3006,6 +3006,9 @@
                 <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
                 <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -3042,6 +3045,23 @@
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2ec83a8d-0db2-4f0a-a71c-c237315b29ff" elementFormDefault="qualified">
@@ -3179,7 +3199,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DB51D13-93B9-40F2-A05B-0E9B0D9A7AA0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF19BC8-7ABF-4D46-B3F6-CA03D9F418A1}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
adaptar scripts para añadir perfil antioquia desde consolar
</commit_message>
<xml_diff>
--- a/Descripcion_fuentes.xlsx
+++ b/Descripcion_fuentes.xlsx
@@ -2990,10 +2990,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010072D1BA84C54EAF45AC5884A45A375563" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e7d927febeb335f2d1c85a73b8edbe09">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="909962d2-3dca-4f1f-a40d-c5b9a956a4cc" xmlns:ns3="2ec83a8d-0db2-4f0a-a71c-c237315b29ff" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="26a6144809e82f96be1dd4a023cacbb7" ns2:_="" ns3:_="">
-    <xsd:import namespace="909962d2-3dca-4f1f-a40d-c5b9a956a4cc"/>
-    <xsd:import namespace="2ec83a8d-0db2-4f0a-a71c-c237315b29ff"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100505E9F3EF18BC1479B9711EB89301B7B" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="2120fe3de92ed2f29333ccc3e6604426">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5781ca24-93bb-44ac-aa4e-2dc5be3c879c" xmlns:ns3="cdc8d142-2086-430e-a051-fd2166eb4d41" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="63cfc21fffc6435508f3aa5d7acc5c9d" ns2:_="" ns3:_="">
+    <xsd:import namespace="5781ca24-93bb-44ac-aa4e-2dc5be3c879c"/>
+    <xsd:import namespace="cdc8d142-2086-430e-a051-fd2166eb4d41"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -3016,7 +3016,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="909962d2-3dca-4f1f-a40d-c5b9a956a4cc" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5781ca24-93bb-44ac-aa4e-2dc5be3c879c" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -3064,10 +3064,10 @@
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="2ec83a8d-0db2-4f0a-a71c-c237315b29ff" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="cdc8d142-2086-430e-a051-fd2166eb4d41" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{2381563d-0fc0-4f9d-9053-aea4d2a325e5}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="2ec83a8d-0db2-4f0a-a71c-c237315b29ff">
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{90c0841c-22ba-4267-b108-7687ee6e2a81}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="cdc8d142-2086-430e-a051-fd2166eb4d41">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:MultiChoiceLookup">
@@ -3190,16 +3190,16 @@
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="909962d2-3dca-4f1f-a40d-c5b9a956a4cc">
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5781ca24-93bb-44ac-aa4e-2dc5be3c879c">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="2ec83a8d-0db2-4f0a-a71c-c237315b29ff" xsi:nil="true"/>
+    <TaxCatchAll xmlns="cdc8d142-2086-430e-a051-fd2166eb4d41" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CBF19BC8-7ABF-4D46-B3F6-CA03D9F418A1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D45873EB-F3E2-44B0-BCF0-3E4A1262C161}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>